<commit_message>
Extend decision threshold grid below 0.001 and recompute threshold-based results
- threshold grid: 0.001-0.999 with step 0.001 plus 20 log steps down to 1e-5
- only IEEE-CIS LightGBM (none, SMOTE) thresholds change; ULB and Sparkov unchanged
- results README: threshold note updated
</commit_message>
<xml_diff>
--- a/experiments/results/results_all.xlsx
+++ b/experiments/results/results_all.xlsx
@@ -2141,7 +2141,7 @@
         <v>0.4917176768897542</v>
       </c>
       <c r="H7">
-        <v>0.5213774438535631</v>
+        <v>0.5213774438535632</v>
       </c>
       <c r="I7">
         <v>0.9019402674513388</v>
@@ -2227,10 +2227,10 @@
         <v>0.531412413725713</v>
       </c>
       <c r="G8">
-        <v>0.516403000160904</v>
+        <v>0.5164030001609039</v>
       </c>
       <c r="H8">
-        <v>0.5463964718315738</v>
+        <v>0.5463964718315737</v>
       </c>
       <c r="I8">
         <v>0.913720041263256</v>
@@ -2402,7 +2402,7 @@
         <v>0.5975322764955009</v>
       </c>
       <c r="G10">
-        <v>0.5825858162318458</v>
+        <v>0.5825858162318459</v>
       </c>
       <c r="H10">
         <v>0.613010670814332</v>
@@ -2491,10 +2491,10 @@
         <v>0.6156126473879366</v>
       </c>
       <c r="G11">
-        <v>0.6010273029137583</v>
+        <v>0.6010273029137582</v>
       </c>
       <c r="H11">
-        <v>0.6299746385790546</v>
+        <v>0.6299746385790547</v>
       </c>
       <c r="I11">
         <v>0.930767459434085</v>
@@ -2580,10 +2580,10 @@
         <v>0.6219294132273525</v>
       </c>
       <c r="G12">
-        <v>0.6078603101589681</v>
+        <v>0.607860310158968</v>
       </c>
       <c r="H12">
-        <v>0.6364394274560783</v>
+        <v>0.6364394274560784</v>
       </c>
       <c r="I12">
         <v>0.9291231748393424</v>
@@ -2669,7 +2669,7 @@
         <v>0.6038269586245321</v>
       </c>
       <c r="G13">
-        <v>0.5886035349245777</v>
+        <v>0.5886035349245776</v>
       </c>
       <c r="H13">
         <v>0.6188663151963667</v>
@@ -2755,46 +2755,46 @@
         <v>0.6341223548031081</v>
       </c>
       <c r="G14">
-        <v>0.6201578126166447</v>
+        <v>0.6201578126166446</v>
       </c>
       <c r="H14">
-        <v>0.6483785154048628</v>
+        <v>0.648378515404863</v>
       </c>
       <c r="I14">
         <v>0.9229310681683296</v>
       </c>
       <c r="J14">
-        <v>0.001</v>
+        <v>0.00063096</v>
       </c>
       <c r="K14">
-        <v>0.3152219873150105</v>
+        <v>0.2704336399474376</v>
       </c>
       <c r="L14">
-        <v>0.7337598425196851</v>
+        <v>0.7595964566929134</v>
       </c>
       <c r="M14">
-        <v>0.4409937888198758</v>
+        <v>0.3988629756444214</v>
       </c>
       <c r="N14">
-        <v>0.579794680354643</v>
+        <v>0.5578041993422717</v>
       </c>
       <c r="O14">
-        <v>0.4545878761305643</v>
+        <v>0.4235388404276528</v>
       </c>
       <c r="P14">
-        <v>0.0568026375784784</v>
+        <v>0.0730244467047806</v>
       </c>
       <c r="Q14">
-        <v>2982</v>
+        <v>3087</v>
       </c>
       <c r="R14">
-        <v>6478</v>
+        <v>8328</v>
       </c>
       <c r="S14">
-        <v>1082</v>
+        <v>977</v>
       </c>
       <c r="T14">
-        <v>107566</v>
+        <v>105716</v>
       </c>
       <c r="U14">
         <v>0.8852370689655172</v>
@@ -2933,46 +2933,46 @@
         <v>0.6330358369239295</v>
       </c>
       <c r="G16">
-        <v>0.6183182948333241</v>
+        <v>0.618318294833324</v>
       </c>
       <c r="H16">
-        <v>0.6474651064276872</v>
+        <v>0.6474651064276874</v>
       </c>
       <c r="I16">
         <v>0.9251051873765672</v>
       </c>
       <c r="J16">
-        <v>0.001</v>
+        <v>0.00063096</v>
       </c>
       <c r="K16">
-        <v>0.3351277058756156</v>
+        <v>0.2918678771489279</v>
       </c>
       <c r="L16">
-        <v>0.71998031496063</v>
+        <v>0.7436023622047244</v>
       </c>
       <c r="M16">
-        <v>0.4573661586557249</v>
+        <v>0.4191982244416701</v>
       </c>
       <c r="N16">
-        <v>0.5855044623204066</v>
+        <v>0.5678316422397595</v>
       </c>
       <c r="O16">
-        <v>0.4661175041223552</v>
+        <v>0.4378357142001664</v>
       </c>
       <c r="P16">
-        <v>0.0509014064746939</v>
+        <v>0.0642909754129985</v>
       </c>
       <c r="Q16">
-        <v>2926</v>
+        <v>3022</v>
       </c>
       <c r="R16">
-        <v>5805</v>
+        <v>7332</v>
       </c>
       <c r="S16">
-        <v>1138</v>
+        <v>1042</v>
       </c>
       <c r="T16">
-        <v>108239</v>
+        <v>106712</v>
       </c>
       <c r="U16">
         <v>0.8774783934926284</v>
@@ -3022,10 +3022,10 @@
         <v>0.627213167706459</v>
       </c>
       <c r="G17">
-        <v>0.6124251386364536</v>
+        <v>0.6124251386364538</v>
       </c>
       <c r="H17">
-        <v>0.642043442149265</v>
+        <v>0.6420434421492651</v>
       </c>
       <c r="I17">
         <v>0.9235192705702482</v>
@@ -3108,7 +3108,7 @@
         <v>0.4833383378633777</v>
       </c>
       <c r="G18">
-        <v>0.4676945622921807</v>
+        <v>0.4676945622921806</v>
       </c>
       <c r="H18">
         <v>0.4984596861400389</v>
@@ -3197,10 +3197,10 @@
         <v>0.4585619444751148</v>
       </c>
       <c r="G19">
-        <v>0.4430369679210048</v>
+        <v>0.4430369679210046</v>
       </c>
       <c r="H19">
-        <v>0.473767134090445</v>
+        <v>0.4737671340904449</v>
       </c>
       <c r="I19">
         <v>0.8775521936881248</v>
@@ -3286,7 +3286,7 @@
         <v>0.4869426877987335</v>
       </c>
       <c r="G20">
-        <v>0.4711442714553949</v>
+        <v>0.471144271455395</v>
       </c>
       <c r="H20">
         <v>0.5016451030645511</v>
@@ -3378,7 +3378,7 @@
         <v>0.4564279925945614</v>
       </c>
       <c r="H21">
-        <v>0.4879525049960722</v>
+        <v>0.4879525049960723</v>
       </c>
       <c r="I21">
         <v>0.8525644444076979</v>
@@ -3566,7 +3566,7 @@
         <v>113680</v>
       </c>
       <c r="P2">
-        <v>0.5929574915130231</v>
+        <v>0.592957491513023</v>
       </c>
       <c r="Q2">
         <v>0.6233910460986948</v>
@@ -3631,7 +3631,7 @@
         <v>107804</v>
       </c>
       <c r="P3">
-        <v>0.5929574915130231</v>
+        <v>0.592957491513023</v>
       </c>
       <c r="Q3">
         <v>0.6233910460986948</v>
@@ -3826,7 +3826,7 @@
         <v>113803</v>
       </c>
       <c r="P6">
-        <v>0.6182281480989608</v>
+        <v>0.6182281480989609</v>
       </c>
       <c r="Q6">
         <v>0.6475086953541553</v>
@@ -3852,7 +3852,7 @@
         <v>117</v>
       </c>
       <c r="C7">
-        <v>0.001</v>
+        <v>0.00063096</v>
       </c>
       <c r="D7">
         <v>0.6330358369239295</v>
@@ -3861,52 +3861,52 @@
         <v>0.9251051873765672</v>
       </c>
       <c r="F7">
-        <v>0.3351277058756156</v>
+        <v>0.2918678771489279</v>
       </c>
       <c r="G7">
-        <v>0.71998031496063</v>
+        <v>0.7436023622047244</v>
       </c>
       <c r="H7">
-        <v>0.4573661586557249</v>
+        <v>0.4191982244416701</v>
       </c>
       <c r="I7">
-        <v>0.5855044623204066</v>
+        <v>0.5678316422397595</v>
       </c>
       <c r="J7">
-        <v>0.4661175041223552</v>
+        <v>0.4378357142001664</v>
       </c>
       <c r="K7">
-        <v>0.0509014064746939</v>
+        <v>0.0642909754129985</v>
       </c>
       <c r="L7">
-        <v>2926</v>
+        <v>3022</v>
       </c>
       <c r="M7">
-        <v>5805</v>
+        <v>7332</v>
       </c>
       <c r="N7">
-        <v>1138</v>
+        <v>1042</v>
       </c>
       <c r="O7">
-        <v>108239</v>
+        <v>106712</v>
       </c>
       <c r="P7">
-        <v>0.6182281480989608</v>
+        <v>0.6182281480989609</v>
       </c>
       <c r="Q7">
         <v>0.6475086953541553</v>
       </c>
       <c r="R7">
-        <v>0.5746780118545801</v>
+        <v>0.5576388131230779</v>
       </c>
       <c r="S7">
-        <v>0.5961385431529241</v>
+        <v>0.5774973251288583</v>
       </c>
       <c r="T7">
-        <v>0.4564150039304325</v>
+        <v>0.4288015052742788</v>
       </c>
       <c r="U7">
-        <v>0.4756511620574148</v>
+        <v>0.4462367323484204</v>
       </c>
     </row>
   </sheetData>
@@ -3965,22 +3965,22 @@
         <v>-0.0314146018383142</v>
       </c>
       <c r="D2">
-        <v>-0.0186960684190574</v>
+        <v>-0.0186960684190576</v>
       </c>
       <c r="E2">
         <v>0.0005</v>
       </c>
       <c r="F2">
-        <v>-0.0182916266344227</v>
+        <v>-0.0006707266588736</v>
       </c>
       <c r="G2">
-        <v>0.0005</v>
+        <v>0.88</v>
       </c>
       <c r="H2">
-        <v>-0.01975876918387</v>
+        <v>0.008460253035938</v>
       </c>
       <c r="I2">
-        <v>0.0005</v>
+        <v>0.036</v>
       </c>
       <c r="J2">
         <v>-0.0002194531320554</v>
@@ -3997,7 +3997,7 @@
         <v>-0.008029306098962999</v>
       </c>
       <c r="C3">
-        <v>-0.0110666438189623</v>
+        <v>-0.0110666438189621</v>
       </c>
       <c r="D3">
         <v>-0.0049743428302064</v>
@@ -4147,19 +4147,19 @@
         <v>0.2587794067908286</v>
       </c>
       <c r="F2">
-        <v>0.2856713576087702</v>
+        <v>0.2856713576087704</v>
       </c>
       <c r="G2">
         <v>0.0005</v>
       </c>
       <c r="H2">
-        <v>0.1890498190209912</v>
+        <v>0.1714296280363452</v>
       </c>
       <c r="I2">
         <v>0.0005</v>
       </c>
       <c r="J2">
-        <v>0.1679317511049278</v>
+        <v>0.1396767387687308</v>
       </c>
       <c r="K2">
         <v>0.0005</v>
@@ -4197,22 +4197,22 @@
         <v>0.2814302703864865</v>
       </c>
       <c r="E3">
-        <v>0.267805845476641</v>
+        <v>0.2678058454766411</v>
       </c>
       <c r="F3">
-        <v>0.2959352604255861</v>
+        <v>0.295935260425586</v>
       </c>
       <c r="G3">
         <v>0.0005</v>
       </c>
       <c r="H3">
-        <v>0.1813978124323043</v>
+        <v>0.1637776214476584</v>
       </c>
       <c r="I3">
         <v>0.0005</v>
       </c>
       <c r="J3">
-        <v>0.1586085178637705</v>
+        <v>0.1303535055275734</v>
       </c>
       <c r="K3">
         <v>0.0005</v>
@@ -4250,22 +4250,22 @@
         <v>0.2697327765308458</v>
       </c>
       <c r="E4">
-        <v>0.2563478060828838</v>
+        <v>0.2563478060828839</v>
       </c>
       <c r="F4">
-        <v>0.2840249741783319</v>
+        <v>0.2840249741783324</v>
       </c>
       <c r="G4">
         <v>0.0005</v>
       </c>
       <c r="H4">
-        <v>0.1792560977266306</v>
+        <v>0.1616359067419847</v>
       </c>
       <c r="I4">
         <v>0.0005</v>
       </c>
       <c r="J4">
-        <v>0.1453025043208379</v>
+        <v>0.1170474919846408</v>
       </c>
       <c r="K4">
         <v>0.0005</v>
@@ -4303,22 +4303,22 @@
         <v>0.2680884195166563</v>
       </c>
       <c r="E5">
-        <v>0.2548776475182387</v>
+        <v>0.2548776475182386</v>
       </c>
       <c r="F5">
-        <v>0.2819686077661613</v>
+        <v>0.2819686077661612</v>
       </c>
       <c r="G5">
         <v>0.0005</v>
       </c>
       <c r="H5">
-        <v>0.1835983734049046</v>
+        <v>0.1659781824202587</v>
       </c>
       <c r="I5">
         <v>0.0005</v>
       </c>
       <c r="J5">
-        <v>0.1581576096614258</v>
+        <v>0.1299025973252287</v>
       </c>
       <c r="K5">
         <v>0.0005</v>
@@ -4359,19 +4359,19 @@
         <v>0.09718825607410091</v>
       </c>
       <c r="F6">
-        <v>0.115314767653268</v>
+        <v>0.1153147676532679</v>
       </c>
       <c r="G6">
         <v>0.0005</v>
       </c>
       <c r="H6">
-        <v>0.0739526671880255</v>
+        <v>0.0563324762033796</v>
       </c>
       <c r="I6">
         <v>0.0005</v>
       </c>
       <c r="J6">
-        <v>0.0753394493002235</v>
+        <v>0.0470844369640264</v>
       </c>
       <c r="K6">
         <v>0.0005</v>
@@ -4412,19 +4412,19 @@
         <v>0.1161933690846535</v>
       </c>
       <c r="F7">
-        <v>0.1380774134785867</v>
+        <v>0.1380774134785868</v>
       </c>
       <c r="G7">
         <v>0.0005</v>
       </c>
       <c r="H7">
-        <v>0.0710229481358661</v>
+        <v>0.0534027571512202</v>
       </c>
       <c r="I7">
         <v>0.0005</v>
       </c>
       <c r="J7">
-        <v>0.0486400006788933</v>
+        <v>0.0203849883426962</v>
       </c>
       <c r="K7">
         <v>0.0005</v>
@@ -4462,22 +4462,22 @@
         <v>0.1015998205835032</v>
       </c>
       <c r="E8">
-        <v>0.0925981169257062</v>
+        <v>0.0925981169257061</v>
       </c>
       <c r="F8">
-        <v>0.110996701301417</v>
+        <v>0.1109967013014172</v>
       </c>
       <c r="G8">
         <v>0.0005</v>
       </c>
       <c r="H8">
-        <v>0.06948455947745399</v>
+        <v>0.051864368492808</v>
       </c>
       <c r="I8">
         <v>0.0005</v>
       </c>
       <c r="J8">
-        <v>0.06673439875509241</v>
+        <v>0.0384793864188953</v>
       </c>
       <c r="K8">
         <v>0.0005</v>
@@ -4515,22 +4515,22 @@
         <v>0.0936291491044156</v>
       </c>
       <c r="E9">
-        <v>0.0847063808045026</v>
+        <v>0.0847063808045025</v>
       </c>
       <c r="F9">
-        <v>0.1027368806242919</v>
+        <v>0.1027368806242917</v>
       </c>
       <c r="G9">
         <v>0.0005</v>
       </c>
       <c r="H9">
-        <v>0.0624519705997988</v>
+        <v>0.0448317796151529</v>
       </c>
       <c r="I9">
         <v>0.0005</v>
       </c>
       <c r="J9">
-        <v>0.0641833708349286</v>
+        <v>0.0359283584987315</v>
       </c>
       <c r="K9">
         <v>0.0005</v>
@@ -4577,16 +4577,16 @@
         <v>0.0005</v>
       </c>
       <c r="H10">
-        <v>0.0153652453265938</v>
+        <v>-0.002254945658052</v>
       </c>
       <c r="I10">
+        <v>0.5679999999999999</v>
+      </c>
+      <c r="J10">
+        <v>-0.0220653632852707</v>
+      </c>
+      <c r="K10">
         <v>0.0005</v>
-      </c>
-      <c r="J10">
-        <v>0.0061896490509263</v>
-      </c>
-      <c r="K10">
-        <v>0.083</v>
       </c>
       <c r="L10">
         <v>0.0052723544314433</v>
@@ -4598,10 +4598,10 @@
         <v>0.0095</v>
       </c>
       <c r="O10">
+        <v>0.5679999999999999</v>
+      </c>
+      <c r="P10">
         <v>0.0095</v>
-      </c>
-      <c r="P10">
-        <v>0.083</v>
       </c>
       <c r="Q10">
         <v>0.0014149096087679</v>
@@ -4621,7 +4621,7 @@
         <v>0.0174641304472984</v>
       </c>
       <c r="E11">
-        <v>0.0120810786547386</v>
+        <v>0.0120810786547387</v>
       </c>
       <c r="F11">
         <v>0.0229064041325363</v>
@@ -4630,13 +4630,13 @@
         <v>0.0005</v>
       </c>
       <c r="H11">
-        <v>-0.0116595357989655</v>
+        <v>-0.0292797267836114</v>
       </c>
       <c r="I11">
-        <v>0.005</v>
+        <v>0.0005</v>
       </c>
       <c r="J11">
-        <v>-0.0289940128032087</v>
+        <v>-0.0572490251394058</v>
       </c>
       <c r="K11">
         <v>0.0005</v>
@@ -4651,7 +4651,7 @@
         <v>0.0095</v>
       </c>
       <c r="O11">
-        <v>0.025</v>
+        <v>0.0095</v>
       </c>
       <c r="P11">
         <v>0.0095</v>
@@ -4677,19 +4677,19 @@
         <v>0.0058021429948975</v>
       </c>
       <c r="F12">
-        <v>0.0163015238679602</v>
+        <v>0.0163015238679603</v>
       </c>
       <c r="G12">
         <v>0.0005</v>
       </c>
       <c r="H12">
-        <v>-0.0056720361987121</v>
+        <v>-0.023292227183358</v>
       </c>
       <c r="I12">
-        <v>0.154</v>
+        <v>0.0005</v>
       </c>
       <c r="J12">
-        <v>-0.0239914479416236</v>
+        <v>-0.0522464602778207</v>
       </c>
       <c r="K12">
         <v>0.0005</v>
@@ -4704,7 +4704,7 @@
         <v>0.0095</v>
       </c>
       <c r="O12">
-        <v>0.4379999999999999</v>
+        <v>0.0095</v>
       </c>
       <c r="P12">
         <v>0.0095</v>
@@ -4727,22 +4727,22 @@
         <v>0.0292615026432469</v>
       </c>
       <c r="E13">
-        <v>0.0234847655897519</v>
+        <v>0.023484765589752</v>
       </c>
       <c r="F13">
-        <v>0.0348297310912975</v>
+        <v>0.0348297310912976</v>
       </c>
       <c r="G13">
         <v>0.0005</v>
       </c>
       <c r="H13">
-        <v>0.001182195217257</v>
+        <v>-0.0164379957673888</v>
       </c>
       <c r="I13">
-        <v>0.793</v>
+        <v>0.0005</v>
       </c>
       <c r="J13">
-        <v>-0.0210141892417252</v>
+        <v>-0.0492692015779223</v>
       </c>
       <c r="K13">
         <v>0.0005</v>
@@ -4757,7 +4757,7 @@
         <v>0.0095</v>
       </c>
       <c r="O13">
-        <v>0.793</v>
+        <v>0.0095</v>
       </c>
       <c r="P13">
         <v>0.0095</v>
@@ -4780,22 +4780,22 @@
         <v>-0.0011009136254431</v>
       </c>
       <c r="E14">
-        <v>-0.0063408521688755</v>
+        <v>-0.0063408521688753</v>
       </c>
       <c r="F14">
-        <v>0.0041270446276079</v>
+        <v>0.0041270446276081</v>
       </c>
       <c r="G14">
         <v>0.681</v>
       </c>
       <c r="H14">
-        <v>0.0056691470258465</v>
+        <v>0.0100557823806698</v>
       </c>
       <c r="I14">
-        <v>0.146</v>
+        <v>0.004</v>
       </c>
       <c r="J14">
-        <v>0.0115077021853261</v>
+        <v>0.0143266012937651</v>
       </c>
       <c r="K14">
         <v>0.0005</v>
@@ -4810,7 +4810,7 @@
         <v>0.681</v>
       </c>
       <c r="O14">
-        <v>0.4379999999999999</v>
+        <v>0.012</v>
       </c>
       <c r="P14">
         <v>0.0095</v>
@@ -4833,22 +4833,22 @@
         <v>0.0065816030563844</v>
       </c>
       <c r="E15">
-        <v>0.0014203998102148</v>
+        <v>0.0014203998102147</v>
       </c>
       <c r="F15">
-        <v>0.0117638004545345</v>
+        <v>0.0117638004545346</v>
       </c>
       <c r="G15">
         <v>0.017</v>
       </c>
       <c r="H15">
-        <v>0.0065514482463731</v>
+        <v>-0.0110687427382727</v>
       </c>
       <c r="I15">
-        <v>0.075</v>
+        <v>0.002</v>
       </c>
       <c r="J15">
-        <v>0.017083090465174</v>
+        <v>-0.011171921871023</v>
       </c>
       <c r="K15">
         <v>0.0005</v>
@@ -4863,7 +4863,7 @@
         <v>0.051</v>
       </c>
       <c r="O15">
-        <v>0.3</v>
+        <v>0.0095</v>
       </c>
       <c r="P15">
         <v>0.0095</v>
@@ -4886,7 +4886,7 @@
         <v>0.0058118387557399</v>
       </c>
       <c r="E16">
-        <v>0.0008089261600428</v>
+        <v>0.0008089261600427</v>
       </c>
       <c r="F16">
         <v>0.0106986005015104</v>
@@ -4895,16 +4895,16 @@
         <v>0.026</v>
       </c>
       <c r="H16">
-        <v>0.0134091674427377</v>
+        <v>-0.0042110235419081</v>
       </c>
       <c r="I16">
-        <v>0.0005</v>
+        <v>0.204</v>
       </c>
       <c r="J16">
-        <v>0.0241066170457609</v>
+        <v>-0.0041483952904361</v>
       </c>
       <c r="K16">
-        <v>0.0005</v>
+        <v>0.181</v>
       </c>
       <c r="L16">
         <v>0.0015859168063189</v>
@@ -4916,10 +4916,10 @@
         <v>0.052</v>
       </c>
       <c r="O16">
-        <v>0.0095</v>
+        <v>0.408</v>
       </c>
       <c r="P16">
-        <v>0.0095</v>
+        <v>0.181</v>
       </c>
       <c r="Q16">
         <v>0.6513630676265271</v>
@@ -4939,25 +4939,25 @@
         <v>0.1497396462371876</v>
       </c>
       <c r="E17">
-        <v>0.1388464227640098</v>
+        <v>0.13884642276401</v>
       </c>
       <c r="F17">
-        <v>0.1604882148254142</v>
+        <v>0.1604882148254144</v>
       </c>
       <c r="G17">
         <v>0.0005</v>
       </c>
       <c r="H17">
-        <v>0.0894949946692386</v>
+        <v>0.0718748036845927</v>
       </c>
       <c r="I17">
         <v>0.0005</v>
       </c>
       <c r="J17">
-        <v>0.0437476823032221</v>
+        <v>0.015492669967025</v>
       </c>
       <c r="K17">
-        <v>0.0005</v>
+        <v>0.002</v>
       </c>
       <c r="L17">
         <v>0.0538199134858708</v>
@@ -4992,7 +4992,7 @@
         <v>0.1744966454251063</v>
       </c>
       <c r="E18">
-        <v>0.1622099960447263</v>
+        <v>0.1622099960447267</v>
       </c>
       <c r="F18">
         <v>0.1863407764742617</v>
@@ -5001,16 +5001,16 @@
         <v>0.0005</v>
       </c>
       <c r="H18">
-        <v>0.09427493637164069</v>
+        <v>0.0766547453869947</v>
       </c>
       <c r="I18">
         <v>0.0005</v>
       </c>
       <c r="J18">
-        <v>0.0428091233392033</v>
+        <v>0.0145541110030062</v>
       </c>
       <c r="K18">
-        <v>0.0005</v>
+        <v>0.008</v>
       </c>
       <c r="L18">
         <v>0.0475529936884423</v>
@@ -5025,7 +5025,7 @@
         <v>0.0095</v>
       </c>
       <c r="P18">
-        <v>0.0095</v>
+        <v>0.024</v>
       </c>
       <c r="Q18">
         <v>1.513395430659441E-67</v>
@@ -5042,25 +5042,25 @@
         <v>75</v>
       </c>
       <c r="D19">
-        <v>0.1462476296806859</v>
+        <v>0.1462476296806858</v>
       </c>
       <c r="E19">
         <v>0.1349718848210671</v>
       </c>
       <c r="F19">
-        <v>0.1577711308860171</v>
+        <v>0.1577711308860172</v>
       </c>
       <c r="G19">
         <v>0.0005</v>
       </c>
       <c r="H19">
-        <v>0.1108607341827344</v>
+        <v>0.0932405431980885</v>
       </c>
       <c r="I19">
         <v>0.0005</v>
       </c>
       <c r="J19">
-        <v>0.0750673277277398</v>
+        <v>0.0468123153915427</v>
       </c>
       <c r="K19">
         <v>0.0005</v>
@@ -5095,28 +5095,28 @@
         <v>76</v>
       </c>
       <c r="D20">
-        <v>0.1607816521796551</v>
+        <v>0.1607816521796552</v>
       </c>
       <c r="E20">
         <v>0.150115312140405</v>
       </c>
       <c r="F20">
-        <v>0.1718180438566413</v>
+        <v>0.1718180438566412</v>
       </c>
       <c r="G20">
         <v>0.0005</v>
       </c>
       <c r="H20">
-        <v>0.1042183315365627</v>
+        <v>0.08659814055191679</v>
       </c>
       <c r="I20">
         <v>0.0005</v>
       </c>
       <c r="J20">
-        <v>0.0160922728696181</v>
+        <v>-0.0121627394665789</v>
       </c>
       <c r="K20">
-        <v>0.005</v>
+        <v>0.042</v>
       </c>
       <c r="L20">
         <v>0.0725407429688692</v>
@@ -5131,7 +5131,7 @@
         <v>0.0095</v>
       </c>
       <c r="P20">
-        <v>0.01</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="Q20">
         <v>5.169864455884663E-108</v>
@@ -5199,7 +5199,7 @@
         <v>-0.009150642019961601</v>
       </c>
       <c r="D2">
-        <v>-0.0141796958712211</v>
+        <v>-0.0141796958712212</v>
       </c>
       <c r="E2">
         <v>-0.0040779440590957</v>
@@ -5223,7 +5223,7 @@
         <v>0.0075</v>
       </c>
       <c r="L2">
-        <v>0.098</v>
+        <v>0.06</v>
       </c>
       <c r="M2">
         <v>1.787169754226603E-13</v>
@@ -5264,7 +5264,7 @@
         <v>0.8370000000000001</v>
       </c>
       <c r="L3">
-        <v>0.018</v>
+        <v>0.014</v>
       </c>
       <c r="M3">
         <v>1.336872407617248E-22</v>
@@ -5284,7 +5284,7 @@
         <v>0.0025615739949214</v>
       </c>
       <c r="E4">
-        <v>0.0057043976998867</v>
+        <v>0.0057043976998866</v>
       </c>
       <c r="F4">
         <v>0.0005</v>
@@ -5305,7 +5305,7 @@
         <v>0.0075</v>
       </c>
       <c r="L4">
-        <v>0.024</v>
+        <v>0.018</v>
       </c>
       <c r="M4">
         <v>4.285434972600985E-13</v>
@@ -5322,10 +5322,10 @@
         <v>-0.0204960444756534</v>
       </c>
       <c r="D5">
-        <v>-0.0267736293213309</v>
+        <v>-0.0267736293213307</v>
       </c>
       <c r="E5">
-        <v>-0.0143888132777523</v>
+        <v>-0.0143888132777526</v>
       </c>
       <c r="F5">
         <v>0.0005</v>
@@ -5346,7 +5346,7 @@
         <v>0.0075</v>
       </c>
       <c r="L5">
-        <v>0.952</v>
+        <v>0.6060000000000001</v>
       </c>
       <c r="M5">
         <v>0.0020533389146279</v>
@@ -5363,7 +5363,7 @@
         <v>0.0046394889392458</v>
       </c>
       <c r="D6">
-        <v>-0.0007712798179642</v>
+        <v>-0.0007712798179641</v>
       </c>
       <c r="E6">
         <v>0.0098165005295316</v>
@@ -5387,7 +5387,7 @@
         <v>0.348</v>
       </c>
       <c r="L6">
-        <v>0.8080000000000001</v>
+        <v>0.6060000000000001</v>
       </c>
       <c r="M6">
         <v>9.632066898686685E-09</v>
@@ -5404,10 +5404,10 @@
         <v>0.0125709034851751</v>
       </c>
       <c r="D7">
-        <v>0.009126157697731899</v>
+        <v>0.0091261576977318</v>
       </c>
       <c r="E7">
-        <v>0.015867519129319</v>
+        <v>0.0158675191293188</v>
       </c>
       <c r="F7">
         <v>0.0005</v>
@@ -5445,10 +5445,10 @@
         <v>0.0180012975357321</v>
       </c>
       <c r="D8">
-        <v>0.0127813494006469</v>
+        <v>0.0127813494006468</v>
       </c>
       <c r="E8">
-        <v>0.0232288887432489</v>
+        <v>0.023228888743249</v>
       </c>
       <c r="F8">
         <v>0.0005</v>
@@ -5489,7 +5489,7 @@
         <v>0.0188494506754562</v>
       </c>
       <c r="E9">
-        <v>0.0295699549447273</v>
+        <v>0.0295699549447272</v>
       </c>
       <c r="F9">
         <v>0.0005</v>
@@ -5527,10 +5527,10 @@
         <v>0.0062656799838276</v>
       </c>
       <c r="D10">
-        <v>0.0006682575687572999</v>
+        <v>0.0006682575687574</v>
       </c>
       <c r="E10">
-        <v>0.0119214887304022</v>
+        <v>0.0119214887304023</v>
       </c>
       <c r="F10">
         <v>0.025</v>
@@ -5568,19 +5568,19 @@
         <v>-0.0077059617713414</v>
       </c>
       <c r="D11">
-        <v>-0.0125240868301625</v>
+        <v>-0.0125240868301624</v>
       </c>
       <c r="E11">
-        <v>-0.0030088590826402</v>
+        <v>-0.0030088590826403</v>
       </c>
       <c r="F11">
         <v>0.002</v>
       </c>
       <c r="G11">
-        <v>-0.0009776664871593999</v>
+        <v>0.0210298207282416</v>
       </c>
       <c r="H11">
-        <v>0.775</v>
+        <v>0.0005</v>
       </c>
       <c r="I11">
         <v>0.0038371394488023</v>
@@ -5592,7 +5592,7 @@
         <v>0.016</v>
       </c>
       <c r="L11">
-        <v>0.952</v>
+        <v>0.0075</v>
       </c>
       <c r="M11">
         <v>0.0112354961307999</v>
@@ -5609,19 +5609,19 @@
         <v>-0.0011469647056722</v>
       </c>
       <c r="D12">
-        <v>-0.0064913805314958</v>
+        <v>-0.0064913805314959</v>
       </c>
       <c r="E12">
-        <v>0.0042941004538633</v>
+        <v>0.0042941004538632</v>
       </c>
       <c r="F12">
         <v>0.658</v>
       </c>
       <c r="G12">
-        <v>0.0054832315733732</v>
+        <v>0.009812442424784301</v>
       </c>
       <c r="H12">
-        <v>0.141</v>
+        <v>0.003</v>
       </c>
       <c r="I12">
         <v>0.0021741192082376</v>
@@ -5633,7 +5633,7 @@
         <v>0.952</v>
       </c>
       <c r="L12">
-        <v>0.705</v>
+        <v>0.018</v>
       </c>
       <c r="M12">
         <v>0.2608414877276774</v>
@@ -5650,7 +5650,7 @@
         <v>-0.0069562855671129</v>
       </c>
       <c r="D13">
-        <v>-0.0120379041564482</v>
+        <v>-0.0120379041564481</v>
       </c>
       <c r="E13">
         <v>-0.0017317879689269</v>
@@ -5659,10 +5659,10 @@
         <v>0.006</v>
       </c>
       <c r="G13">
-        <v>-0.0077571068675644</v>
+        <v>0.0142503803478366</v>
       </c>
       <c r="H13">
-        <v>0.014</v>
+        <v>0.0005</v>
       </c>
       <c r="I13">
         <v>0.0005882024019187001</v>
@@ -5674,7 +5674,7 @@
         <v>0.036</v>
       </c>
       <c r="L13">
-        <v>0.098</v>
+        <v>0.0075</v>
       </c>
       <c r="M13">
         <v>0.6616745433673734</v>
@@ -5694,7 +5694,7 @@
         <v>-0.03029788357346</v>
       </c>
       <c r="E14">
-        <v>-0.0191502444565815</v>
+        <v>-0.0191502444565813</v>
       </c>
       <c r="F14">
         <v>0.0005</v>
@@ -5715,7 +5715,7 @@
         <v>0.0075</v>
       </c>
       <c r="L14">
-        <v>0.8080000000000001</v>
+        <v>0.6060000000000001</v>
       </c>
       <c r="M14">
         <v>0.0016507682384292</v>
@@ -5732,10 +5732,10 @@
         <v>0.0036375352887848</v>
       </c>
       <c r="D15">
-        <v>-0.006838040380662</v>
+        <v>-0.0068380403806621</v>
       </c>
       <c r="E15">
-        <v>0.0143066438570593</v>
+        <v>0.0143066438570592</v>
       </c>
       <c r="F15">
         <v>0.476</v>
@@ -5776,7 +5776,7 @@
         <v>-0.0176495424685594</v>
       </c>
       <c r="E16">
-        <v>-0.0040080585876788</v>
+        <v>-0.0040080585876789</v>
       </c>
       <c r="F16">
         <v>0.002</v>
@@ -5850,19 +5850,19 @@
         <v>0.9112781954887216</v>
       </c>
       <c r="D2">
-        <v>0.6090225563909774</v>
+        <v>0.4661654135338345</v>
       </c>
       <c r="E2">
-        <v>0.9203007518796992</v>
+        <v>0.8812030075187969</v>
       </c>
       <c r="F2">
-        <v>0.7639097744360903</v>
+        <v>0.7022556390977444</v>
       </c>
       <c r="G2">
-        <v>0.3864661654135338</v>
+        <v>0.3172932330827067</v>
       </c>
       <c r="H2">
-        <v>0.9548872180451128</v>
+        <v>0.9624060150375938</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -5876,19 +5876,19 @@
         <v>1</v>
       </c>
       <c r="D3">
-        <v>0.7293233082706766</v>
+        <v>0.6541353383458646</v>
       </c>
       <c r="E3">
-        <v>0.9834586466165413</v>
+        <v>0.9804511278195488</v>
       </c>
       <c r="F3">
-        <v>0.8556390977443609</v>
+        <v>0.8270676691729323</v>
       </c>
       <c r="G3">
-        <v>0.5293233082706766</v>
+        <v>0.4977443609022556</v>
       </c>
       <c r="H3">
-        <v>0.9067669172932332</v>
+        <v>0.8992481203007519</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -5896,25 +5896,25 @@
         <v>51</v>
       </c>
       <c r="B4">
-        <v>0.6090225563909774</v>
+        <v>0.4661654135338345</v>
       </c>
       <c r="C4">
-        <v>0.7293233082706766</v>
+        <v>0.6541353383458646</v>
       </c>
       <c r="D4">
         <v>1</v>
       </c>
       <c r="E4">
-        <v>0.7624060150375939</v>
+        <v>0.7037593984962407</v>
       </c>
       <c r="F4">
-        <v>0.9669172932330824</v>
+        <v>0.9293233082706768</v>
       </c>
       <c r="G4">
-        <v>0.9413533834586464</v>
+        <v>0.9654135338345864</v>
       </c>
       <c r="H4">
-        <v>0.5293233082706766</v>
+        <v>0.4240601503759398</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -5922,25 +5922,25 @@
         <v>52</v>
       </c>
       <c r="B5">
-        <v>0.9203007518796992</v>
+        <v>0.8812030075187969</v>
       </c>
       <c r="C5">
-        <v>0.9834586466165413</v>
+        <v>0.9804511278195488</v>
       </c>
       <c r="D5">
-        <v>0.7624060150375939</v>
+        <v>0.7037593984962407</v>
       </c>
       <c r="E5">
         <v>1</v>
       </c>
       <c r="F5">
-        <v>0.882706766917293</v>
+        <v>0.8601503759398496</v>
       </c>
       <c r="G5">
-        <v>0.5624060150375939</v>
+        <v>0.5548872180451127</v>
       </c>
       <c r="H5">
-        <v>0.8902255639097743</v>
+        <v>0.8736842105263156</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -5948,25 +5948,25 @@
         <v>53</v>
       </c>
       <c r="B6">
-        <v>0.7639097744360903</v>
+        <v>0.7022556390977444</v>
       </c>
       <c r="C6">
-        <v>0.8556390977443609</v>
+        <v>0.8270676691729323</v>
       </c>
       <c r="D6">
-        <v>0.9669172932330824</v>
+        <v>0.9293233082706768</v>
       </c>
       <c r="E6">
-        <v>0.882706766917293</v>
+        <v>0.8601503759398496</v>
       </c>
       <c r="F6">
         <v>1</v>
       </c>
       <c r="G6">
-        <v>0.8421052631578947</v>
+        <v>0.8330827067669173</v>
       </c>
       <c r="H6">
-        <v>0.6977443609022556</v>
+        <v>0.6571428571428571</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -5974,25 +5974,25 @@
         <v>49</v>
       </c>
       <c r="B7">
-        <v>0.3864661654135338</v>
+        <v>0.3172932330827067</v>
       </c>
       <c r="C7">
-        <v>0.5293233082706766</v>
+        <v>0.4977443609022556</v>
       </c>
       <c r="D7">
-        <v>0.9413533834586464</v>
+        <v>0.9654135338345864</v>
       </c>
       <c r="E7">
-        <v>0.5624060150375939</v>
+        <v>0.5548872180451127</v>
       </c>
       <c r="F7">
-        <v>0.8421052631578947</v>
+        <v>0.8330827067669173</v>
       </c>
       <c r="G7">
         <v>1</v>
       </c>
       <c r="H7">
-        <v>0.3037593984962406</v>
+        <v>0.2556390977443609</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -6000,22 +6000,22 @@
         <v>50</v>
       </c>
       <c r="B8">
-        <v>0.9548872180451128</v>
+        <v>0.9624060150375938</v>
       </c>
       <c r="C8">
-        <v>0.9067669172932332</v>
+        <v>0.8992481203007519</v>
       </c>
       <c r="D8">
-        <v>0.5293233082706766</v>
+        <v>0.4240601503759398</v>
       </c>
       <c r="E8">
-        <v>0.8902255639097743</v>
+        <v>0.8736842105263156</v>
       </c>
       <c r="F8">
-        <v>0.6977443609022556</v>
+        <v>0.6571428571428571</v>
       </c>
       <c r="G8">
-        <v>0.3037593984962406</v>
+        <v>0.2556390977443609</v>
       </c>
       <c r="H8">
         <v>1</v>
@@ -6876,7 +6876,7 @@
         <v>0.1694301186532323</v>
       </c>
       <c r="F37">
-        <v>0.001</v>
+        <v>1E-05</v>
       </c>
       <c r="G37" t="b">
         <v>0</v>
@@ -7320,10 +7320,10 @@
         <v>0.7910623502665266</v>
       </c>
       <c r="G2">
-        <v>0.7021138736406838</v>
+        <v>0.7021138736406837</v>
       </c>
       <c r="H2">
-        <v>0.8735985759009451</v>
+        <v>0.8735985759009453</v>
       </c>
       <c r="I2">
         <v>0.9792500848886718</v>
@@ -7409,7 +7409,7 @@
         <v>0.8020737738497823</v>
       </c>
       <c r="G3">
-        <v>0.7126399007526941</v>
+        <v>0.712639900752694</v>
       </c>
       <c r="H3">
         <v>0.8835953039445223</v>
@@ -7587,10 +7587,10 @@
         <v>0.786839686939359</v>
       </c>
       <c r="G5">
-        <v>0.6910035308140019</v>
+        <v>0.691003530814002</v>
       </c>
       <c r="H5">
-        <v>0.8738869699123476</v>
+        <v>0.8738869699123475</v>
       </c>
       <c r="I5">
         <v>0.9845685032505684</v>
@@ -7673,10 +7673,10 @@
         <v>0.7968938509539253</v>
       </c>
       <c r="G6">
-        <v>0.7067050959902202</v>
+        <v>0.7067050959902204</v>
       </c>
       <c r="H6">
-        <v>0.880144593907654</v>
+        <v>0.8801445939076541</v>
       </c>
       <c r="I6">
         <v>0.971590193736933</v>
@@ -7762,10 +7762,10 @@
         <v>0.7828966357369537</v>
       </c>
       <c r="G7">
-        <v>0.6923008076326223</v>
+        <v>0.6923008076326225</v>
       </c>
       <c r="H7">
-        <v>0.8668378003292465</v>
+        <v>0.8668378003292467</v>
       </c>
       <c r="I7">
         <v>0.987594092893006</v>
@@ -7854,7 +7854,7 @@
         <v>0.7110250256898988</v>
       </c>
       <c r="H8">
-        <v>0.8793523700720371</v>
+        <v>0.8793523700720373</v>
       </c>
       <c r="I8">
         <v>0.986538945778076</v>
@@ -8026,10 +8026,10 @@
         <v>0.8043384608749143</v>
       </c>
       <c r="G10">
-        <v>0.7136865009703454</v>
+        <v>0.7136865009703456</v>
       </c>
       <c r="H10">
-        <v>0.8880615037460121</v>
+        <v>0.8880615037460122</v>
       </c>
       <c r="I10">
         <v>0.9906631999023304</v>
@@ -8115,7 +8115,7 @@
         <v>0.7926019228438927</v>
       </c>
       <c r="G11">
-        <v>0.7023882529314105</v>
+        <v>0.7023882529314106</v>
       </c>
       <c r="H11">
         <v>0.8778273654141748</v>
@@ -8207,7 +8207,7 @@
         <v>0.7128578078205411</v>
       </c>
       <c r="H12">
-        <v>0.883042581634102</v>
+        <v>0.8830425816341021</v>
       </c>
       <c r="I12">
         <v>0.9838294233674668</v>
@@ -8293,10 +8293,10 @@
         <v>0.7926681980828018</v>
       </c>
       <c r="G13">
-        <v>0.7012174477660327</v>
+        <v>0.7012174477660329</v>
       </c>
       <c r="H13">
-        <v>0.8758820312305334</v>
+        <v>0.8758820312305335</v>
       </c>
       <c r="I13">
         <v>0.9780236104964366</v>
@@ -8379,7 +8379,7 @@
         <v>0.8120647931143029</v>
       </c>
       <c r="G14">
-        <v>0.725389677798742</v>
+        <v>0.7253896777987422</v>
       </c>
       <c r="H14">
         <v>0.8928161262629899</v>
@@ -8468,7 +8468,7 @@
         <v>0.7597329407664318</v>
       </c>
       <c r="G15">
-        <v>0.6659992657951113</v>
+        <v>0.6659992657951114</v>
       </c>
       <c r="H15">
         <v>0.8477744022473072</v>
@@ -8649,7 +8649,7 @@
         <v>0.7124786402905027</v>
       </c>
       <c r="H17">
-        <v>0.8849518806782198</v>
+        <v>0.8849518806782199</v>
       </c>
       <c r="I17">
         <v>0.9857205808292764</v>
@@ -8735,7 +8735,7 @@
         <v>0.7269659939538913</v>
       </c>
       <c r="H18">
-        <v>0.8953673897533194</v>
+        <v>0.8953673897533192</v>
       </c>
       <c r="I18">
         <v>0.9865241617959007</v>
@@ -8910,7 +8910,7 @@
         <v>0.7478603066622147</v>
       </c>
       <c r="G20">
-        <v>0.6497918078930489</v>
+        <v>0.6497918078930488</v>
       </c>
       <c r="H20">
         <v>0.8437903216309126</v>
@@ -8999,7 +8999,7 @@
         <v>0.7646716673916607</v>
       </c>
       <c r="G21">
-        <v>0.673582315876024</v>
+        <v>0.6735823158760241</v>
       </c>
       <c r="H21">
         <v>0.8555535487727244</v>
@@ -14226,7 +14226,7 @@
         <v>0.0252355711833811</v>
       </c>
       <c r="F31">
-        <v>0.001</v>
+        <v>1E-05</v>
       </c>
       <c r="G31" t="b">
         <v>0</v>
@@ -14249,7 +14249,7 @@
         <v>0.0252355711833811</v>
       </c>
       <c r="F32">
-        <v>0.001</v>
+        <v>1E-05</v>
       </c>
       <c r="G32" t="b">
         <v>0</v>
@@ -14272,7 +14272,7 @@
         <v>0.0252355711833811</v>
       </c>
       <c r="F33">
-        <v>0.001</v>
+        <v>1E-05</v>
       </c>
       <c r="G33" t="b">
         <v>0</v>
@@ -14295,7 +14295,7 @@
         <v>0.0252355711833811</v>
       </c>
       <c r="F34">
-        <v>0.001</v>
+        <v>1E-05</v>
       </c>
       <c r="G34" t="b">
         <v>0</v>
@@ -14341,7 +14341,7 @@
         <v>0.0252355711833811</v>
       </c>
       <c r="F36">
-        <v>0.001</v>
+        <v>1E-05</v>
       </c>
       <c r="G36" t="b">
         <v>0</v>
@@ -15744,7 +15744,7 @@
         <v>56672</v>
       </c>
       <c r="P2">
-        <v>0.7341491391111555</v>
+        <v>0.7341491391111559</v>
       </c>
       <c r="Q2">
         <v>0.8943768486656565</v>
@@ -15809,7 +15809,7 @@
         <v>56660</v>
       </c>
       <c r="P3">
-        <v>0.7341491391111555</v>
+        <v>0.7341491391111559</v>
       </c>
       <c r="Q3">
         <v>0.8943768486656565</v>
@@ -15874,7 +15874,7 @@
         <v>56670</v>
       </c>
       <c r="P4">
-        <v>0.7355036266216733</v>
+        <v>0.7355036266216732</v>
       </c>
       <c r="Q4">
         <v>0.8955379957772701</v>
@@ -15939,7 +15939,7 @@
         <v>56658</v>
       </c>
       <c r="P5">
-        <v>0.7355036266216733</v>
+        <v>0.7355036266216732</v>
       </c>
       <c r="Q5">
         <v>0.8955379957772701</v>
@@ -16004,10 +16004,10 @@
         <v>56670</v>
       </c>
       <c r="P6">
-        <v>0.7169393956305111</v>
+        <v>0.7169393956305113</v>
       </c>
       <c r="Q6">
-        <v>0.8848029022551148</v>
+        <v>0.8848029022551149</v>
       </c>
       <c r="R6">
         <v>0.685131195335277</v>
@@ -16069,10 +16069,10 @@
         <v>56652</v>
       </c>
       <c r="P7">
-        <v>0.7169393956305111</v>
+        <v>0.7169393956305113</v>
       </c>
       <c r="Q7">
-        <v>0.8848029022551148</v>
+        <v>0.8848029022551149</v>
       </c>
       <c r="R7">
         <v>0.6910340089316386</v>
@@ -18092,10 +18092,10 @@
         <v>-0.0016738177037676</v>
       </c>
       <c r="C3">
-        <v>-0.0042237559264642</v>
+        <v>-0.004223755926464</v>
       </c>
       <c r="D3">
-        <v>0.0003283365483403</v>
+        <v>0.0003283365483402</v>
       </c>
       <c r="E3">
         <v>0.1</v>
@@ -18239,10 +18239,10 @@
         <v>0.0129965784087466</v>
       </c>
       <c r="E2">
-        <v>-0.0162079256446709</v>
+        <v>-0.016207925644671</v>
       </c>
       <c r="F2">
-        <v>0.0481922270691059</v>
+        <v>0.048192227069106</v>
       </c>
       <c r="G2">
         <v>0.416</v>
@@ -18292,10 +18292,10 @@
         <v>0.0022102185770029</v>
       </c>
       <c r="E3">
-        <v>-0.0219784576724643</v>
+        <v>-0.0219784576724645</v>
       </c>
       <c r="F3">
-        <v>0.0264667870221987</v>
+        <v>0.0264667870221988</v>
       </c>
       <c r="G3">
         <v>0.847</v>
@@ -18342,10 +18342,10 @@
         <v>75</v>
       </c>
       <c r="D4">
-        <v>0.026383617991274</v>
+        <v>0.0263836179912741</v>
       </c>
       <c r="E4">
-        <v>-0.0100023947509709</v>
+        <v>-0.010002394750971</v>
       </c>
       <c r="F4">
         <v>0.0759425443976541</v>
@@ -18395,7 +18395,7 @@
         <v>76</v>
       </c>
       <c r="D5">
-        <v>0.0172372874252933</v>
+        <v>0.0172372874252934</v>
       </c>
       <c r="E5">
         <v>-0.0151287942541953</v>
@@ -18454,7 +18454,7 @@
         <v>-0.0181368464000176</v>
       </c>
       <c r="F6">
-        <v>0.035314940834019</v>
+        <v>0.0353149408340192</v>
       </c>
       <c r="G6">
         <v>0.623</v>
@@ -18504,7 +18504,7 @@
         <v>0.0212361066178371</v>
       </c>
       <c r="E7">
-        <v>-0.0078605047887107</v>
+        <v>-0.007860504788710801</v>
       </c>
       <c r="F7">
         <v>0.0529051831479931</v>
@@ -18557,10 +18557,10 @@
         <v>0.0046711826838843</v>
       </c>
       <c r="E8">
-        <v>-0.0222960943902082</v>
+        <v>-0.0222960943902087</v>
       </c>
       <c r="F8">
-        <v>0.0325756205922274</v>
+        <v>0.0325756205922275</v>
       </c>
       <c r="G8">
         <v>0.74</v>
@@ -18610,10 +18610,10 @@
         <v>-0.0118034196115792</v>
       </c>
       <c r="E9">
-        <v>-0.0375718551034344</v>
+        <v>-0.0375718551034346</v>
       </c>
       <c r="F9">
-        <v>0.0124798776708766</v>
+        <v>0.0124798776708767</v>
       </c>
       <c r="G9">
         <v>0.362</v>
@@ -18663,10 +18663,10 @@
         <v>0.0119040576619617</v>
       </c>
       <c r="E10">
-        <v>-0.0217040667581363</v>
+        <v>-0.0217040667581364</v>
       </c>
       <c r="F10">
-        <v>0.0462261692725058</v>
+        <v>0.046226169272506</v>
       </c>
       <c r="G10">
         <v>0.482</v>
@@ -18716,10 +18716,10 @@
         <v>0.0027807696740383</v>
       </c>
       <c r="E11">
-        <v>-0.0154548548722444</v>
+        <v>-0.0154548548722445</v>
       </c>
       <c r="F11">
-        <v>0.0206593410993849</v>
+        <v>0.020659341099385</v>
       </c>
       <c r="G11">
         <v>0.736</v>
@@ -18766,13 +18766,13 @@
         <v>76</v>
       </c>
       <c r="D12">
-        <v>0.011445036652166</v>
+        <v>0.0114450366521661</v>
       </c>
       <c r="E12">
-        <v>-0.008629193788373599</v>
+        <v>-0.0086291937883737</v>
       </c>
       <c r="F12">
-        <v>0.0331674678853152</v>
+        <v>0.0331674678853154</v>
       </c>
       <c r="G12">
         <v>0.283</v>
@@ -18822,7 +18822,7 @@
         <v>-0.0078844989609765</v>
       </c>
       <c r="E13">
-        <v>-0.0187379407347013</v>
+        <v>-0.0187379407347012</v>
       </c>
       <c r="F13">
         <v>0.002028451293117</v>
@@ -18931,7 +18931,7 @@
         <v>-0.0104789010804876</v>
       </c>
       <c r="F15">
-        <v>0.0266406911816002</v>
+        <v>0.0266406911816003</v>
       </c>
       <c r="G15">
         <v>0.379</v>
@@ -18978,10 +18978,10 @@
         <v>76</v>
       </c>
       <c r="D16">
-        <v>0.0025305478766819</v>
+        <v>0.002530547876682</v>
       </c>
       <c r="E16">
-        <v>-0.0227448260055465</v>
+        <v>-0.0227448260055466</v>
       </c>
       <c r="F16">
         <v>0.0285387971030978</v>
@@ -19034,10 +19034,10 @@
         <v>-0.0099871311269414</v>
       </c>
       <c r="E17">
-        <v>-0.0358857656001629</v>
+        <v>-0.0358857656001628</v>
       </c>
       <c r="F17">
-        <v>0.0137103728463491</v>
+        <v>0.0137103728463489</v>
       </c>
       <c r="G17">
         <v>0.428</v>
@@ -19084,7 +19084,7 @@
         <v>74</v>
       </c>
       <c r="D18">
-        <v>0.0144836746191722</v>
+        <v>0.0144836746191723</v>
       </c>
       <c r="E18">
         <v>-0.0115359403217075</v>
@@ -19140,7 +19140,7 @@
         <v>0.0554202341693246</v>
       </c>
       <c r="E19">
-        <v>0.0157878917378396</v>
+        <v>0.0157878917378397</v>
       </c>
       <c r="F19">
         <v>0.1054584752565978</v>
@@ -19190,13 +19190,13 @@
         <v>76</v>
       </c>
       <c r="D20">
-        <v>0.0385361286640091</v>
+        <v>0.0385361286640092</v>
       </c>
       <c r="E20">
-        <v>0.0035732138364988</v>
+        <v>0.0035732138364985</v>
       </c>
       <c r="F20">
-        <v>0.08159122991639869</v>
+        <v>0.08159122991639881</v>
       </c>
       <c r="G20">
         <v>0.029</v>
@@ -19291,7 +19291,7 @@
         <v>74</v>
       </c>
       <c r="C2">
-        <v>0.0106351695177177</v>
+        <v>0.0106351695177178</v>
       </c>
       <c r="D2">
         <v>-0.0075521862922945</v>
@@ -19335,10 +19335,10 @@
         <v>-0.0130626101410308</v>
       </c>
       <c r="D3">
-        <v>-0.0377482739789019</v>
+        <v>-0.037748273978902</v>
       </c>
       <c r="E3">
-        <v>0.0061447103579801</v>
+        <v>0.00614471035798</v>
       </c>
       <c r="F3">
         <v>0.227</v>
@@ -19376,10 +19376,10 @@
         <v>-0.0039042300706189</v>
       </c>
       <c r="D4">
-        <v>-0.0262882879184554</v>
+        <v>-0.0262882879184555</v>
       </c>
       <c r="E4">
-        <v>0.0164218926895973</v>
+        <v>0.0164218926895972</v>
       </c>
       <c r="F4">
         <v>0.726</v>
@@ -19420,7 +19420,7 @@
         <v>-0.0424574339070282</v>
       </c>
       <c r="E5">
-        <v>0.0140113454834082</v>
+        <v>0.0140113454834083</v>
       </c>
       <c r="F5">
         <v>0.312</v>
@@ -19458,7 +19458,7 @@
         <v>0.0020205204732799</v>
       </c>
       <c r="D6">
-        <v>-0.0188042783055991</v>
+        <v>-0.0188042783055988</v>
       </c>
       <c r="E6">
         <v>0.0231796381694175</v>
@@ -19499,10 +19499,10 @@
         <v>0.0188480081640287</v>
       </c>
       <c r="D7">
-        <v>-0.0068437582839369</v>
+        <v>-0.006843758283937</v>
       </c>
       <c r="E7">
-        <v>0.0467289130085532</v>
+        <v>0.0467289130085534</v>
       </c>
       <c r="F7">
         <v>0.141</v>
@@ -19543,7 +19543,7 @@
         <v>-0.0465200844069661</v>
       </c>
       <c r="E8">
-        <v>0.0216111479962851</v>
+        <v>0.0216111479962852</v>
       </c>
       <c r="F8">
         <v>0.461</v>
@@ -19578,13 +19578,13 @@
         <v>75</v>
       </c>
       <c r="C9">
-        <v>-0.0027567489472777</v>
+        <v>-0.0027567489472778</v>
       </c>
       <c r="D9">
-        <v>-0.0200780399587685</v>
+        <v>-0.0200780399587686</v>
       </c>
       <c r="E9">
-        <v>0.0166654574408327</v>
+        <v>0.0166654574408325</v>
       </c>
       <c r="F9">
         <v>0.741</v>
@@ -19619,13 +19619,13 @@
         <v>76</v>
       </c>
       <c r="C10">
-        <v>-0.0112197495615475</v>
+        <v>-0.0112197495615476</v>
       </c>
       <c r="D10">
         <v>-0.0323888615944625</v>
       </c>
       <c r="E10">
-        <v>0.0090824604184182</v>
+        <v>0.009082460418418301</v>
       </c>
       <c r="F10">
         <v>0.285</v>
@@ -19663,10 +19663,10 @@
         <v>-0.0525806791252687</v>
       </c>
       <c r="D11">
-        <v>-0.1031360238032773</v>
+        <v>-0.1031360238032772</v>
       </c>
       <c r="E11">
-        <v>-0.008962289508403901</v>
+        <v>-0.008962289508403999</v>
       </c>
       <c r="F11">
         <v>0.013</v>
@@ -19701,10 +19701,10 @@
         <v>75</v>
       </c>
       <c r="C12">
-        <v>-0.0159367766072352</v>
+        <v>-0.0159367766072353</v>
       </c>
       <c r="D12">
-        <v>-0.0342501473809284</v>
+        <v>-0.0342501473809282</v>
       </c>
       <c r="E12">
         <v>-0.0004272810047212</v>
@@ -19745,7 +19745,7 @@
         <v>-0.0102731624740552</v>
       </c>
       <c r="D13">
-        <v>-0.0346617550081668</v>
+        <v>-0.0346617550081672</v>
       </c>
       <c r="E13">
         <v>0.0103523886470962</v>
@@ -19786,7 +19786,7 @@
         <v>-0.0245610466148798</v>
       </c>
       <c r="D14">
-        <v>-0.0466314583707985</v>
+        <v>-0.0466314583707987</v>
       </c>
       <c r="E14">
         <v>-0.0068714145167537</v>
@@ -19865,13 +19865,13 @@
         <v>76</v>
       </c>
       <c r="C16">
-        <v>-0.0494028782287003</v>
+        <v>-0.0494028782287004</v>
       </c>
       <c r="D16">
-        <v>-0.0879331889659152</v>
+        <v>-0.0879331889659155</v>
       </c>
       <c r="E16">
-        <v>-0.0188842289517182</v>
+        <v>-0.0188842289517181</v>
       </c>
       <c r="F16">
         <v>0.0005</v>
@@ -20488,7 +20488,7 @@
         <v>0.0070640031541595</v>
       </c>
       <c r="F16">
-        <v>0.001</v>
+        <v>1E-05</v>
       </c>
       <c r="G16" t="b">
         <v>0</v>
@@ -20511,7 +20511,7 @@
         <v>0.0070640031541595</v>
       </c>
       <c r="F17">
-        <v>0.001</v>
+        <v>1E-05</v>
       </c>
       <c r="G17" t="b">
         <v>0</v>
@@ -20672,7 +20672,7 @@
         <v>0.0070640031541595</v>
       </c>
       <c r="F24">
-        <v>0.001</v>
+        <v>1E-05</v>
       </c>
       <c r="G24" t="b">
         <v>0</v>
@@ -20695,7 +20695,7 @@
         <v>0.0070640031541595</v>
       </c>
       <c r="F25">
-        <v>0.001</v>
+        <v>1E-05</v>
       </c>
       <c r="G25" t="b">
         <v>0</v>
@@ -20856,7 +20856,7 @@
         <v>0.0070640031541595</v>
       </c>
       <c r="F32">
-        <v>0.001</v>
+        <v>1E-05</v>
       </c>
       <c r="G32" t="b">
         <v>0</v>

</xml_diff>